<commit_message>
Experiment complete for lottery scheduling
</commit_message>
<xml_diff>
--- a/Metrics.xlsx
+++ b/Metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pankajsharma/Downloads/AOS Lab 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pankajsharma/Desktop/Masters/Spring 2025/xv6-riscv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B84B46F-4AEB-C647-89C7-B32655EF7367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31FA5B0-5B84-124F-961D-4E11933FF70C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="3" xr2:uid="{4F434C4C-E251-CC45-9265-F0D894057F2F}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21100" activeTab="3" xr2:uid="{4F434C4C-E251-CC45-9265-F0D894057F2F}"/>
   </bookViews>
   <sheets>
     <sheet name="STRIDE (8 4 2 1)" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="LOTTERY (8 4 2 1)" sheetId="5" r:id="rId3"/>
     <sheet name="LOTTERY (1 1 1 1)" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -124,7 +124,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2144,18 +2165,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E18145CB-2816-5C46-8F37-F37C74845109}">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2172,37 +2193,117 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <f>SUM(B4:E4)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>19</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <f t="shared" ref="F5:F8" si="0">SUM(B5:E5)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>60</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>30</v>
+      </c>
+      <c r="C6">
+        <v>17</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>80</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>38</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
+      </c>
+      <c r="D7">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>100</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>54</v>
+      </c>
+      <c r="C8">
+        <v>27</v>
+      </c>
+      <c r="D8">
+        <v>13</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -2219,37 +2320,117 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>9</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F5:F61" si="1">SUM(B13:E13)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>40</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>17</v>
+      </c>
+      <c r="C14">
+        <v>14</v>
+      </c>
+      <c r="D14">
+        <v>6</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>60</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>32</v>
+      </c>
+      <c r="C15">
+        <v>15</v>
+      </c>
+      <c r="D15">
+        <v>9</v>
+      </c>
+      <c r="E15">
+        <v>4</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>80</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <v>45</v>
+      </c>
+      <c r="C16">
+        <v>14</v>
+      </c>
+      <c r="D16">
+        <v>17</v>
+      </c>
+      <c r="E16">
+        <v>4</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>100</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B17">
+        <v>68</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>13</v>
+      </c>
+      <c r="E17">
+        <v>5</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="1"/>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -2266,37 +2447,117 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>13</v>
+      </c>
+      <c r="C22">
+        <v>4</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>40</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>22</v>
+      </c>
+      <c r="C23">
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>5</v>
+      </c>
+      <c r="E23">
+        <v>3</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>60</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>33</v>
+      </c>
+      <c r="C24">
+        <v>15</v>
+      </c>
+      <c r="D24">
+        <v>10</v>
+      </c>
+      <c r="E24">
+        <v>2</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>80</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>38</v>
+      </c>
+      <c r="C25">
+        <v>21</v>
+      </c>
+      <c r="D25">
+        <v>12</v>
+      </c>
+      <c r="E25">
+        <v>9</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>100</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>59</v>
+      </c>
+      <c r="C26">
+        <v>26</v>
+      </c>
+      <c r="D26">
+        <v>11</v>
+      </c>
+      <c r="E26">
+        <v>4</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>5</v>
       </c>
@@ -2313,37 +2574,117 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>20</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B31">
+        <v>9</v>
+      </c>
+      <c r="C31">
+        <v>9</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>40</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B32">
+        <v>15</v>
+      </c>
+      <c r="C32">
+        <v>15</v>
+      </c>
+      <c r="D32">
+        <v>7</v>
+      </c>
+      <c r="E32">
+        <v>3</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>60</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B33">
+        <v>34</v>
+      </c>
+      <c r="C33">
+        <v>15</v>
+      </c>
+      <c r="D33">
+        <v>8</v>
+      </c>
+      <c r="E33">
+        <v>3</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>80</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B34">
+        <v>43</v>
+      </c>
+      <c r="C34">
+        <v>20</v>
+      </c>
+      <c r="D34">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <v>8</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>100</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B35">
+        <v>56</v>
+      </c>
+      <c r="C35">
+        <v>26</v>
+      </c>
+      <c r="D35">
+        <v>13</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>5</v>
       </c>
@@ -2360,32 +2701,112 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>20</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B40">
+        <v>10</v>
+      </c>
+      <c r="C40">
+        <v>4</v>
+      </c>
+      <c r="D40">
+        <v>4</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B41">
+        <v>24</v>
+      </c>
+      <c r="C41">
+        <v>6</v>
+      </c>
+      <c r="D41">
+        <v>7</v>
+      </c>
+      <c r="E41">
+        <v>3</v>
+      </c>
+      <c r="F41">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>60</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B42">
+        <v>30</v>
+      </c>
+      <c r="C42">
+        <v>18</v>
+      </c>
+      <c r="D42">
+        <v>8</v>
+      </c>
+      <c r="E42">
+        <v>4</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>80</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B43">
+        <v>36</v>
+      </c>
+      <c r="C43">
+        <v>25</v>
+      </c>
+      <c r="D43">
+        <v>12</v>
+      </c>
+      <c r="E43">
+        <v>7</v>
+      </c>
+      <c r="F43">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>100</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B44">
+        <v>59</v>
+      </c>
+      <c r="C44">
+        <v>16</v>
+      </c>
+      <c r="D44">
+        <v>21</v>
+      </c>
+      <c r="E44">
+        <v>4</v>
+      </c>
+      <c r="F44">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>10</v>
       </c>
@@ -2394,14 +2815,14 @@
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>5</v>
       </c>
@@ -2418,112 +2839,132 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>20</v>
       </c>
-      <c r="B49" s="1" t="e">
+      <c r="B49" s="1">
         <f>AVERAGE(B4,B13,B22,B31,B40)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C49" s="1" t="e">
+        <v>10.4</v>
+      </c>
+      <c r="C49" s="1">
         <f>AVERAGE(C4,C13,C22,C31,C40)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D49" s="1" t="e">
+        <v>5.6</v>
+      </c>
+      <c r="D49" s="1">
         <f>AVERAGE(D4,D13,D22,D31,D40)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E49" s="1" t="e">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E49" s="1">
         <f>AVERAGE(E4,E13,E22,E31,E40)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1.8</v>
+      </c>
+      <c r="F49">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>40</v>
       </c>
-      <c r="B50" s="1" t="e">
+      <c r="B50" s="1">
         <f>AVERAGE(B5,B14,B23,B32,B41)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C50" s="1" t="e">
-        <f t="shared" ref="C50:E50" si="0">AVERAGE(C5,C14,C23,C32,C41)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D50" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E50" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="C50" s="1">
+        <f t="shared" ref="C50:E50" si="2">AVERAGE(C5,C14,C23,C32,C41)</f>
+        <v>11.2</v>
+      </c>
+      <c r="D50" s="1">
+        <f t="shared" si="2"/>
+        <v>6.6</v>
+      </c>
+      <c r="E50" s="1">
+        <f t="shared" si="2"/>
+        <v>2.8</v>
+      </c>
+      <c r="F50">
+        <f t="shared" si="1"/>
+        <v>39.999999999999993</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>60</v>
       </c>
-      <c r="B51" s="1" t="e">
-        <f t="shared" ref="B51:E53" si="1">AVERAGE(B6,B15,B24,B33,B42)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C51" s="1" t="e">
+      <c r="B51" s="1">
+        <f t="shared" ref="B51:E53" si="3">AVERAGE(B6,B15,B24,B33,B42)</f>
+        <v>31.8</v>
+      </c>
+      <c r="C51" s="1">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="D51" s="1">
+        <f t="shared" si="3"/>
+        <v>7.8</v>
+      </c>
+      <c r="E51" s="1">
+        <f t="shared" si="3"/>
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="F51">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D51" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E51" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+        <v>59.999999999999993</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>80</v>
       </c>
-      <c r="B52" s="1" t="e">
+      <c r="B52" s="1">
+        <f t="shared" si="3"/>
+        <v>40</v>
+      </c>
+      <c r="C52" s="1">
+        <f t="shared" si="3"/>
+        <v>21</v>
+      </c>
+      <c r="D52" s="1">
+        <f>AVERAGE(D7,D16,D25,D34,D43)</f>
+        <v>12.6</v>
+      </c>
+      <c r="E52" s="1">
+        <f t="shared" si="3"/>
+        <v>6.4</v>
+      </c>
+      <c r="F52">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C52" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D52" s="1" t="e">
-        <f>AVERAGE(D7,D16,D25,D34,D43)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E52" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>100</v>
       </c>
-      <c r="B53" s="1" t="e">
+      <c r="B53" s="1">
+        <f t="shared" si="3"/>
+        <v>59.2</v>
+      </c>
+      <c r="C53" s="1">
+        <f t="shared" si="3"/>
+        <v>22.2</v>
+      </c>
+      <c r="D53" s="1">
+        <f>AVERAGE(D8,D17,D26,D35,D44)</f>
+        <v>14.2</v>
+      </c>
+      <c r="E53" s="1">
+        <f t="shared" si="3"/>
+        <v>4.8</v>
+      </c>
+      <c r="F53">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C53" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D53" s="1" t="e">
-        <f>AVERAGE(D8,D17,D26,D35,D44)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E53" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+        <v>100.4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>11</v>
       </c>
@@ -2540,7 +2981,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>20</v>
       </c>
@@ -2556,8 +2997,12 @@
       <c r="E57" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F57">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>40</v>
       </c>
@@ -2566,19 +3011,23 @@
         <v>20</v>
       </c>
       <c r="C58" s="1">
-        <f t="shared" ref="C58:E58" si="2">C57*2</f>
+        <f t="shared" ref="C58:E58" si="4">C57*2</f>
         <v>10</v>
       </c>
       <c r="D58" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="E58" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F58">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>60</v>
       </c>
@@ -2587,19 +3036,23 @@
         <v>30</v>
       </c>
       <c r="C59" s="1">
-        <f t="shared" ref="C59:E59" si="3">C57*3</f>
+        <f t="shared" ref="C59:E59" si="5">C57*3</f>
         <v>15</v>
       </c>
       <c r="D59" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>9</v>
       </c>
       <c r="E59" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F59">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>80</v>
       </c>
@@ -2608,19 +3061,23 @@
         <v>40</v>
       </c>
       <c r="C60" s="1">
-        <f t="shared" ref="C60:E60" si="4">C57*4</f>
+        <f t="shared" ref="C60:E60" si="6">C57*4</f>
         <v>20</v>
       </c>
       <c r="D60" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>12</v>
       </c>
       <c r="E60" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F60">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>100</v>
       </c>
@@ -2629,19 +3086,33 @@
         <v>50</v>
       </c>
       <c r="C61" s="1">
-        <f t="shared" ref="C61:E61" si="5">C57*5</f>
+        <f t="shared" ref="C61:E61" si="7">C57*5</f>
         <v>25</v>
       </c>
       <c r="D61" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>15</v>
       </c>
       <c r="E61" s="1">
-        <f t="shared" si="5"/>
-        <v>10</v>
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="F61">
+        <f t="shared" si="1"/>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F4:F8">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+      <formula>$A$4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F8">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>$A$5</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -2681,46 +3152,86 @@
       <c r="A4">
         <v>20</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
+      <c r="B4" s="1">
+        <v>5</v>
+      </c>
+      <c r="C4" s="1">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1">
+        <v>6</v>
+      </c>
+      <c r="E4" s="1">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>40</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
+      <c r="B5" s="1">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1">
+        <v>7</v>
+      </c>
+      <c r="E5" s="1">
+        <v>14</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>60</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
+      <c r="B6" s="1">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1">
+        <v>16</v>
+      </c>
+      <c r="E6" s="1">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>80</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
+      <c r="B7" s="1">
+        <v>25</v>
+      </c>
+      <c r="C7" s="1">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1">
+        <v>18</v>
+      </c>
+      <c r="E7" s="1">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>100</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="B8" s="1">
+        <v>21</v>
+      </c>
+      <c r="C8" s="1">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1">
+        <v>28</v>
+      </c>
+      <c r="E8" s="1">
+        <v>26</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -2748,46 +3259,86 @@
       <c r="A13">
         <v>20</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+      <c r="B13" s="1">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1">
+        <v>8</v>
+      </c>
+      <c r="D13" s="1">
+        <v>6</v>
+      </c>
+      <c r="E13" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>40</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="B14" s="1">
+        <v>9</v>
+      </c>
+      <c r="C14" s="1">
+        <v>6</v>
+      </c>
+      <c r="D14" s="1">
+        <v>15</v>
+      </c>
+      <c r="E14" s="1">
+        <v>10</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>60</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
+      <c r="B15" s="1">
+        <v>14</v>
+      </c>
+      <c r="C15" s="1">
+        <v>15</v>
+      </c>
+      <c r="D15" s="1">
+        <v>18</v>
+      </c>
+      <c r="E15" s="1">
+        <v>13</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>80</v>
       </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
+      <c r="B16" s="1">
+        <v>19</v>
+      </c>
+      <c r="C16" s="1">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1">
+        <v>25</v>
+      </c>
+      <c r="E16" s="1">
+        <v>21</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>100</v>
       </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
+      <c r="B17" s="1">
+        <v>23</v>
+      </c>
+      <c r="C17" s="1">
+        <v>31</v>
+      </c>
+      <c r="D17" s="1">
+        <v>21</v>
+      </c>
+      <c r="E17" s="1">
+        <v>25</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -2815,46 +3366,86 @@
       <c r="A22">
         <v>20</v>
       </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
+      <c r="B22" s="1">
+        <v>7</v>
+      </c>
+      <c r="C22" s="1">
+        <v>4</v>
+      </c>
+      <c r="D22" s="1">
+        <v>5</v>
+      </c>
+      <c r="E22" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>40</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+      <c r="B23" s="1">
+        <v>6</v>
+      </c>
+      <c r="C23" s="1">
+        <v>10</v>
+      </c>
+      <c r="D23" s="1">
+        <v>14</v>
+      </c>
+      <c r="E23" s="1">
+        <v>10</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>60</v>
       </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
+      <c r="B24" s="1">
+        <v>14</v>
+      </c>
+      <c r="C24" s="1">
+        <v>16</v>
+      </c>
+      <c r="D24" s="1">
+        <v>17</v>
+      </c>
+      <c r="E24" s="1">
+        <v>13</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>80</v>
       </c>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
+      <c r="B25" s="1">
+        <v>22</v>
+      </c>
+      <c r="C25" s="1">
+        <v>22</v>
+      </c>
+      <c r="D25" s="1">
+        <v>20</v>
+      </c>
+      <c r="E25" s="1">
+        <v>16</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>100</v>
       </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
+      <c r="B26" s="1">
+        <v>22</v>
+      </c>
+      <c r="C26" s="1">
+        <v>31</v>
+      </c>
+      <c r="D26" s="1">
+        <v>28</v>
+      </c>
+      <c r="E26" s="1">
+        <v>19</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
@@ -2882,46 +3473,86 @@
       <c r="A31">
         <v>20</v>
       </c>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
+      <c r="B31" s="1">
+        <v>6</v>
+      </c>
+      <c r="C31" s="1">
+        <v>4</v>
+      </c>
+      <c r="D31" s="1">
+        <v>6</v>
+      </c>
+      <c r="E31" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>40</v>
       </c>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
+      <c r="B32" s="1">
+        <v>12</v>
+      </c>
+      <c r="C32" s="1">
+        <v>12</v>
+      </c>
+      <c r="D32" s="1">
+        <v>8</v>
+      </c>
+      <c r="E32" s="1">
+        <v>8</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>60</v>
       </c>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
+      <c r="B33" s="1">
+        <v>14</v>
+      </c>
+      <c r="C33" s="1">
+        <v>12</v>
+      </c>
+      <c r="D33" s="1">
+        <v>16</v>
+      </c>
+      <c r="E33" s="1">
+        <v>18</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>80</v>
       </c>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
+      <c r="B34" s="1">
+        <v>27</v>
+      </c>
+      <c r="C34" s="1">
+        <v>19</v>
+      </c>
+      <c r="D34" s="1">
+        <v>19</v>
+      </c>
+      <c r="E34" s="1">
+        <v>15</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>100</v>
       </c>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
+      <c r="B35" s="1">
+        <v>24</v>
+      </c>
+      <c r="C35" s="1">
+        <v>25</v>
+      </c>
+      <c r="D35" s="1">
+        <v>25</v>
+      </c>
+      <c r="E35" s="1">
+        <v>26</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
@@ -2949,46 +3580,86 @@
       <c r="A40">
         <v>20</v>
       </c>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
+      <c r="B40" s="1">
+        <v>2</v>
+      </c>
+      <c r="C40" s="1">
+        <v>7</v>
+      </c>
+      <c r="D40" s="1">
+        <v>3</v>
+      </c>
+      <c r="E40" s="1">
+        <v>8</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
+      <c r="B41" s="1">
+        <v>6</v>
+      </c>
+      <c r="C41" s="1">
+        <v>9</v>
+      </c>
+      <c r="D41" s="1">
+        <v>7</v>
+      </c>
+      <c r="E41" s="1">
+        <v>18</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>60</v>
       </c>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
+      <c r="B42">
+        <v>9</v>
+      </c>
+      <c r="C42">
+        <v>14</v>
+      </c>
+      <c r="D42">
+        <v>21</v>
+      </c>
+      <c r="E42">
+        <v>16</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>80</v>
       </c>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
+      <c r="B43" s="1">
+        <v>24</v>
+      </c>
+      <c r="C43" s="1">
+        <v>16</v>
+      </c>
+      <c r="D43" s="1">
+        <v>19</v>
+      </c>
+      <c r="E43" s="1">
+        <v>21</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>100</v>
       </c>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
+      <c r="B44" s="1">
+        <v>23</v>
+      </c>
+      <c r="C44" s="1">
+        <v>33</v>
+      </c>
+      <c r="D44" s="1">
+        <v>23</v>
+      </c>
+      <c r="E44" s="1">
+        <v>21</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -3027,105 +3698,105 @@
       <c r="A49" s="1">
         <v>20</v>
       </c>
-      <c r="B49" s="1" t="e">
+      <c r="B49" s="1">
         <f>AVERAGE(B4,B13,B22,B31,B40)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C49" s="1" t="e">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="C49" s="1">
         <f>AVERAGE(C4,C13,C22,C31,C40)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D49" s="1" t="e">
+        <v>5.4</v>
+      </c>
+      <c r="D49" s="1">
         <f>AVERAGE(D4,D13,D22,D31,D40)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E49" s="1" t="e">
+        <v>5.2</v>
+      </c>
+      <c r="E49" s="1">
         <f>AVERAGE(E4,E13,E22,E31,E40)</f>
-        <v>#DIV/0!</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>40</v>
       </c>
-      <c r="B50" s="1" t="e">
+      <c r="B50" s="1">
         <f>AVERAGE(B5,B14,B23,B32,B41)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C50" s="1" t="e">
+        <v>8.6</v>
+      </c>
+      <c r="C50" s="1">
         <f t="shared" ref="C50:E50" si="0">AVERAGE(C5,C14,C23,C32,C41)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D50" s="1" t="e">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="D50" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E50" s="1" t="e">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="E50" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>12</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>60</v>
       </c>
-      <c r="B51" s="1" t="e">
-        <f t="shared" ref="B51:E53" si="1">AVERAGE(B6,B15,B24,B33,B42)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C51" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D51" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E51" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+      <c r="B51" s="1">
+        <f>AVERAGE(B6,B15,B24,B33,B42)</f>
+        <v>13.2</v>
+      </c>
+      <c r="C51" s="1">
+        <f>AVERAGE(C6,C15,C24,C33,C42)</f>
+        <v>14.2</v>
+      </c>
+      <c r="D51" s="1">
+        <f>AVERAGE(D6,D15,D24,D33,D42)</f>
+        <v>17.600000000000001</v>
+      </c>
+      <c r="E51" s="1">
+        <f>AVERAGE(E6,E15,E24,E33,E42)</f>
+        <v>15</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>80</v>
       </c>
-      <c r="B52" s="1" t="e">
+      <c r="B52" s="1">
+        <f t="shared" ref="B51:E53" si="1">AVERAGE(B7,B16,B25,B34,B43)</f>
+        <v>23.4</v>
+      </c>
+      <c r="C52" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C52" s="1" t="e">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="D52" s="1">
+        <f>AVERAGE(D7,D16,D25,D34,D43)</f>
+        <v>20.2</v>
+      </c>
+      <c r="E52" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D52" s="1" t="e">
-        <f>AVERAGE(D7,D16,D25,D34,D43)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E52" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>18</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>100</v>
       </c>
-      <c r="B53" s="1" t="e">
+      <c r="B53" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C53" s="1" t="e">
+        <v>22.6</v>
+      </c>
+      <c r="C53" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D53" s="1" t="e">
+        <v>29</v>
+      </c>
+      <c r="D53" s="1">
         <f>AVERAGE(D8,D17,D26,D35,D44)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E53" s="1" t="e">
+        <v>25</v>
+      </c>
+      <c r="E53" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>